<commit_message>
Eliminar convenio erroneo Puno-Amazonas (Hospital Carlos Monge Medrano -> Santa Maria de Nieva)
El codigo RENIPRESS 3299 en la planilla semaforo pertenece en realidad
al Hospital de Apoyo Gustavo Lanatta Lujan, no al hospital de Puno con
el mismo codigo en el registro nacional; ese cruce generaba un
convenio ficticio de 2546 km. Se retira la fila de la fuente, se
regenera la red de convenios del aplicativo (278 -> 277) y se
actualizan el Excel y la presentacion resumen.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/Convenios_tiempos_ruta_BS2_a_BS1.xlsx
+++ b/datos/Convenios_tiempos_ruta_BS2_a_BS1.xlsx
@@ -441,7 +441,7 @@
         </is>
       </c>
       <c r="L4">
-        <v>1.99891666666667</v>
+        <v>1.9989166666666665</v>
       </c>
       <c r="M4">
         <v>1.5</v>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="L5">
-        <v>3.47083333333333</v>
+        <v>3.4708333333333332</v>
       </c>
       <c r="M5">
         <v>1.5</v>
@@ -621,7 +621,7 @@
         </is>
       </c>
       <c r="L6">
-        <v>0.790833333333333</v>
+        <v>0.79083333333333328</v>
       </c>
       <c r="M6">
         <v>1.5</v>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="L7">
-        <v>1.55141666666667</v>
+        <v>1.5514166666666669</v>
       </c>
       <c r="M7">
         <v>1.5</v>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="L8">
-        <v>2.49397777777778</v>
+        <v>2.4939777777777783</v>
       </c>
       <c r="M8">
         <v>1.12</v>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="L9">
-        <v>0.429848888888889</v>
+        <v>0.42984888888888895</v>
       </c>
       <c r="M9">
         <v>1.12</v>
@@ -1071,7 +1071,7 @@
         </is>
       </c>
       <c r="L11">
-        <v>0.429848888888889</v>
+        <v>0.42984888888888895</v>
       </c>
       <c r="M11">
         <v>1.12</v>
@@ -1161,7 +1161,7 @@
         </is>
       </c>
       <c r="L12">
-        <v>0.429848888888889</v>
+        <v>0.42984888888888895</v>
       </c>
       <c r="M12">
         <v>1.12</v>
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="L13">
-        <v>0.429848888888889</v>
+        <v>0.42984888888888895</v>
       </c>
       <c r="M13">
         <v>1.12</v>
@@ -1431,7 +1431,7 @@
         </is>
       </c>
       <c r="L15">
-        <v>0.429848888888889</v>
+        <v>0.42984888888888895</v>
       </c>
       <c r="M15">
         <v>1.12</v>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="L17">
-        <v>2.77313333333333</v>
+        <v>2.7731333333333335</v>
       </c>
       <c r="M17">
         <v>1.3</v>
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="L18">
-        <v>0.338991666666667</v>
+        <v>0.33899166666666669</v>
       </c>
       <c r="M18">
         <v>1.3</v>
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="L19">
-        <v>2.76793333333333</v>
+        <v>2.7679333333333336</v>
       </c>
       <c r="M19">
         <v>1.3</v>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="L20">
-        <v>0.338991666666667</v>
+        <v>0.33899166666666669</v>
       </c>
       <c r="M20">
         <v>1.3</v>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="L21">
-        <v>0.339063888888889</v>
+        <v>0.33906388888888894</v>
       </c>
       <c r="M21">
         <v>1.3</v>
@@ -2386,7 +2386,7 @@
         </is>
       </c>
       <c r="L27">
-        <v>0.338991666666667</v>
+        <v>0.33899166666666669</v>
       </c>
       <c r="M27">
         <v>1.3</v>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="L28">
-        <v>0.400380555555556</v>
+        <v>0.40038055555555557</v>
       </c>
       <c r="M28">
         <v>1.3</v>
@@ -2566,7 +2566,7 @@
         </is>
       </c>
       <c r="L29">
-        <v>0.342494444444444</v>
+        <v>0.34249444444444443</v>
       </c>
       <c r="M29">
         <v>1.3</v>
@@ -2656,7 +2656,7 @@
         </is>
       </c>
       <c r="L30">
-        <v>0.338991666666667</v>
+        <v>0.33899166666666669</v>
       </c>
       <c r="M30">
         <v>1.3</v>
@@ -2746,7 +2746,7 @@
         </is>
       </c>
       <c r="L31">
-        <v>0.338991666666667</v>
+        <v>0.33899166666666669</v>
       </c>
       <c r="M31">
         <v>1.3</v>
@@ -2836,7 +2836,7 @@
         </is>
       </c>
       <c r="L32">
-        <v>0.398683333333333</v>
+        <v>0.39868333333333339</v>
       </c>
       <c r="M32">
         <v>1.3</v>
@@ -3106,7 +3106,7 @@
         </is>
       </c>
       <c r="L35">
-        <v>4.06111111111111</v>
+        <v>4.0611111111111109</v>
       </c>
       <c r="M35">
         <v>1.3</v>
@@ -3196,7 +3196,7 @@
         </is>
       </c>
       <c r="L36">
-        <v>2.77313333333333</v>
+        <v>2.7731333333333335</v>
       </c>
       <c r="M36">
         <v>1.3</v>
@@ -3286,7 +3286,7 @@
         </is>
       </c>
       <c r="L37">
-        <v>0.426272222222222</v>
+        <v>0.42627222222222227</v>
       </c>
       <c r="M37">
         <v>1.3</v>
@@ -3376,7 +3376,7 @@
         </is>
       </c>
       <c r="L38">
-        <v>0.338991666666667</v>
+        <v>0.33899166666666669</v>
       </c>
       <c r="M38">
         <v>1.3</v>
@@ -3466,7 +3466,7 @@
         </is>
       </c>
       <c r="L39">
-        <v>2.738375</v>
+        <v>2.7383750000000004</v>
       </c>
       <c r="M39">
         <v>1.5</v>
@@ -3556,7 +3556,7 @@
         </is>
       </c>
       <c r="L40">
-        <v>1.49906111111111</v>
+        <v>1.4990611111111112</v>
       </c>
       <c r="M40">
         <v>1.3</v>
@@ -3646,7 +3646,7 @@
         </is>
       </c>
       <c r="L41">
-        <v>6.07008333333333</v>
+        <v>6.0700833333333337</v>
       </c>
       <c r="M41">
         <v>1.5</v>
@@ -3736,7 +3736,7 @@
         </is>
       </c>
       <c r="L42">
-        <v>5.41316666666667</v>
+        <v>5.4131666666666671</v>
       </c>
       <c r="M42">
         <v>1.5</v>
@@ -4006,7 +4006,7 @@
         </is>
       </c>
       <c r="L45">
-        <v>0.626346666666667</v>
+        <v>0.62634666666666683</v>
       </c>
       <c r="M45">
         <v>1.12</v>
@@ -4096,7 +4096,7 @@
         </is>
       </c>
       <c r="L46">
-        <v>0.519511111111111</v>
+        <v>0.51951111111111126</v>
       </c>
       <c r="M46">
         <v>1.12</v>
@@ -4251,7 +4251,7 @@
         </is>
       </c>
       <c r="L48">
-        <v>0.322608888888889</v>
+        <v>0.32260888888888894</v>
       </c>
       <c r="M48">
         <v>1.12</v>
@@ -4341,7 +4341,7 @@
         </is>
       </c>
       <c r="L49">
-        <v>6.95708333333333</v>
+        <v>6.9570833333333333</v>
       </c>
       <c r="M49">
         <v>1.5</v>
@@ -4521,7 +4521,7 @@
         </is>
       </c>
       <c r="L51">
-        <v>4.21866666666667</v>
+        <v>4.2186666666666666</v>
       </c>
       <c r="M51">
         <v>1.5</v>
@@ -4701,7 +4701,7 @@
         </is>
       </c>
       <c r="L53">
-        <v>0.539333333333333</v>
+        <v>0.53933333333333333</v>
       </c>
       <c r="M53">
         <v>1.5</v>
@@ -4791,7 +4791,7 @@
         </is>
       </c>
       <c r="L54">
-        <v>0.306958333333333</v>
+        <v>0.30695833333333333</v>
       </c>
       <c r="M54">
         <v>1.5</v>
@@ -5151,7 +5151,7 @@
         </is>
       </c>
       <c r="L58">
-        <v>6.95708333333333</v>
+        <v>6.9570833333333333</v>
       </c>
       <c r="M58">
         <v>1.5</v>
@@ -5241,7 +5241,7 @@
         </is>
       </c>
       <c r="L59">
-        <v>0.306958333333333</v>
+        <v>0.30695833333333333</v>
       </c>
       <c r="M59">
         <v>1.5</v>
@@ -5331,7 +5331,7 @@
         </is>
       </c>
       <c r="L60">
-        <v>2.26711555555556</v>
+        <v>2.2671155555555562</v>
       </c>
       <c r="M60">
         <v>1.12</v>
@@ -5421,7 +5421,7 @@
         </is>
       </c>
       <c r="L61">
-        <v>2.26711555555556</v>
+        <v>2.2671155555555562</v>
       </c>
       <c r="M61">
         <v>1.12</v>
@@ -5511,7 +5511,7 @@
         </is>
       </c>
       <c r="L62">
-        <v>2.26711555555556</v>
+        <v>2.2671155555555562</v>
       </c>
       <c r="M62">
         <v>1.12</v>
@@ -5601,7 +5601,7 @@
         </is>
       </c>
       <c r="L63">
-        <v>2.26711555555556</v>
+        <v>2.2671155555555562</v>
       </c>
       <c r="M63">
         <v>1.12</v>
@@ -6051,7 +6051,7 @@
         </is>
       </c>
       <c r="L68">
-        <v>3.95783333333333</v>
+        <v>3.9578333333333338</v>
       </c>
       <c r="M68">
         <v>1.5</v>
@@ -6141,7 +6141,7 @@
         </is>
       </c>
       <c r="L69">
-        <v>4.44995833333333</v>
+        <v>4.449958333333333</v>
       </c>
       <c r="M69">
         <v>1.5</v>
@@ -6633,7 +6633,7 @@
         </is>
       </c>
       <c r="L74">
-        <v>0.329416666666667</v>
+        <v>0.32941666666666669</v>
       </c>
       <c r="M74">
         <v>1.5</v>
@@ -6813,7 +6813,7 @@
         </is>
       </c>
       <c r="L76">
-        <v>0.847041666666667</v>
+        <v>0.84704166666666669</v>
       </c>
       <c r="M76">
         <v>1.5</v>
@@ -6903,7 +6903,7 @@
         </is>
       </c>
       <c r="L77">
-        <v>0.847041666666667</v>
+        <v>0.84704166666666669</v>
       </c>
       <c r="M77">
         <v>1.5</v>
@@ -6993,7 +6993,7 @@
         </is>
       </c>
       <c r="L78">
-        <v>0.847041666666667</v>
+        <v>0.84704166666666669</v>
       </c>
       <c r="M78">
         <v>1.5</v>
@@ -7083,7 +7083,7 @@
         </is>
       </c>
       <c r="L79">
-        <v>0.896041666666667</v>
+        <v>0.89604166666666663</v>
       </c>
       <c r="M79">
         <v>1.5</v>
@@ -7243,7 +7243,7 @@
         </is>
       </c>
       <c r="L81">
-        <v>0.847041666666667</v>
+        <v>0.84704166666666669</v>
       </c>
       <c r="M81">
         <v>1.5</v>
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="L82">
-        <v>2.19770833333333</v>
+        <v>2.1977083333333338</v>
       </c>
       <c r="M82">
         <v>1.5</v>
@@ -7568,7 +7568,7 @@
         </is>
       </c>
       <c r="L85">
-        <v>0.350266666666667</v>
+        <v>0.35026666666666667</v>
       </c>
       <c r="M85">
         <v>1.12</v>
@@ -8218,7 +8218,7 @@
         </is>
       </c>
       <c r="L93">
-        <v>0.338071111111111</v>
+        <v>0.3380711111111111</v>
       </c>
       <c r="M93">
         <v>1.12</v>
@@ -8308,7 +8308,7 @@
         </is>
       </c>
       <c r="L94">
-        <v>0.355773333333333</v>
+        <v>0.35577333333333339</v>
       </c>
       <c r="M94">
         <v>1.12</v>
@@ -8398,7 +8398,7 @@
         </is>
       </c>
       <c r="L95">
-        <v>1.80710666666667</v>
+        <v>1.8071066666666664</v>
       </c>
       <c r="M95">
         <v>1.12</v>
@@ -8543,7 +8543,7 @@
         </is>
       </c>
       <c r="L97">
-        <v>0.359568888888889</v>
+        <v>0.35956888888888894</v>
       </c>
       <c r="M97">
         <v>1.12</v>
@@ -8633,7 +8633,7 @@
         </is>
       </c>
       <c r="L98">
-        <v>0.359568888888889</v>
+        <v>0.35956888888888894</v>
       </c>
       <c r="M98">
         <v>1.12</v>
@@ -8723,7 +8723,7 @@
         </is>
       </c>
       <c r="L99">
-        <v>1.85284166666667</v>
+        <v>1.8528416666666669</v>
       </c>
       <c r="M99">
         <v>1.3</v>
@@ -8813,7 +8813,7 @@
         </is>
       </c>
       <c r="L100">
-        <v>1.28636888888889</v>
+        <v>1.2863688888888889</v>
       </c>
       <c r="M100">
         <v>1.12</v>
@@ -8903,7 +8903,7 @@
         </is>
       </c>
       <c r="L101">
-        <v>10.4014711111111</v>
+        <v>10.401471111111114</v>
       </c>
       <c r="M101">
         <v>1.12</v>
@@ -9014,7 +9014,7 @@
         </is>
       </c>
       <c r="L102">
-        <v>0.350266666666667</v>
+        <v>0.35026666666666667</v>
       </c>
       <c r="M102">
         <v>1.12</v>
@@ -9104,7 +9104,7 @@
         </is>
       </c>
       <c r="L103">
-        <v>2.58124444444445</v>
+        <v>2.5812444444444451</v>
       </c>
       <c r="M103">
         <v>1.12</v>
@@ -9485,7 +9485,7 @@
         </is>
       </c>
       <c r="L107">
-        <v>0.466591111111111</v>
+        <v>0.46659111111111118</v>
       </c>
       <c r="M107">
         <v>1.12</v>
@@ -9575,7 +9575,7 @@
         </is>
       </c>
       <c r="L108">
-        <v>1.59984444444444</v>
+        <v>1.5998444444444444</v>
       </c>
       <c r="M108">
         <v>1.12</v>
@@ -9845,7 +9845,7 @@
         </is>
       </c>
       <c r="L111">
-        <v>0.284404444444444</v>
+        <v>0.28440444444444446</v>
       </c>
       <c r="M111">
         <v>1.12</v>
@@ -10475,7 +10475,7 @@
         </is>
       </c>
       <c r="L118">
-        <v>0.439244444444444</v>
+        <v>0.43924444444444449</v>
       </c>
       <c r="M118">
         <v>1.12</v>
@@ -10565,7 +10565,7 @@
         </is>
       </c>
       <c r="L119">
-        <v>0.36212</v>
+        <v>0.36212000000000005</v>
       </c>
       <c r="M119">
         <v>1.12</v>
@@ -10655,7 +10655,7 @@
         </is>
       </c>
       <c r="L120">
-        <v>0.353657777777778</v>
+        <v>0.35365777777777779</v>
       </c>
       <c r="M120">
         <v>1.12</v>
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="L122">
-        <v>0.854111111111111</v>
+        <v>0.85411111111111127</v>
       </c>
       <c r="M122">
         <v>1.12</v>
@@ -11165,7 +11165,7 @@
         </is>
       </c>
       <c r="L126">
-        <v>0.762862222222222</v>
+        <v>0.76286222222222233</v>
       </c>
       <c r="M126">
         <v>1.12</v>
@@ -11255,7 +11255,7 @@
         </is>
       </c>
       <c r="L127">
-        <v>0.375933333333333</v>
+        <v>0.37593333333333334</v>
       </c>
       <c r="M127">
         <v>1.12</v>
@@ -11345,7 +11345,7 @@
         </is>
       </c>
       <c r="L128">
-        <v>0.602235555555556</v>
+        <v>0.60223555555555564</v>
       </c>
       <c r="M128">
         <v>1.12</v>
@@ -11705,7 +11705,7 @@
         </is>
       </c>
       <c r="L133">
-        <v>0.499444444444444</v>
+        <v>0.49944444444444447</v>
       </c>
       <c r="M133">
         <v>1.12</v>
@@ -11795,7 +11795,7 @@
         </is>
       </c>
       <c r="L134">
-        <v>0.757262222222222</v>
+        <v>0.75726222222222228</v>
       </c>
       <c r="M134">
         <v>1.12</v>
@@ -12125,7 +12125,7 @@
         </is>
       </c>
       <c r="L138">
-        <v>0.606591111111111</v>
+        <v>0.60659111111111119</v>
       </c>
       <c r="M138">
         <v>1.12</v>
@@ -12305,7 +12305,7 @@
         </is>
       </c>
       <c r="L140">
-        <v>0.629333333333333</v>
+        <v>0.62933333333333341</v>
       </c>
       <c r="M140">
         <v>1.12</v>
@@ -12395,7 +12395,7 @@
         </is>
       </c>
       <c r="L141">
-        <v>0.523928888888889</v>
+        <v>0.52392888888888889</v>
       </c>
       <c r="M141">
         <v>1.12</v>
@@ -12485,7 +12485,7 @@
         </is>
       </c>
       <c r="L142">
-        <v>0.348368888888889</v>
+        <v>0.34836888888888889</v>
       </c>
       <c r="M142">
         <v>1.12</v>
@@ -12665,7 +12665,7 @@
         </is>
       </c>
       <c r="L144">
-        <v>0.602235555555556</v>
+        <v>0.60223555555555564</v>
       </c>
       <c r="M144">
         <v>1.12</v>
@@ -12755,7 +12755,7 @@
         </is>
       </c>
       <c r="L145">
-        <v>0.499444444444444</v>
+        <v>0.49944444444444447</v>
       </c>
       <c r="M145">
         <v>1.12</v>
@@ -12845,7 +12845,7 @@
         </is>
       </c>
       <c r="L146">
-        <v>0.452373333333333</v>
+        <v>0.45237333333333341</v>
       </c>
       <c r="M146">
         <v>1.12</v>
@@ -12935,7 +12935,7 @@
         </is>
       </c>
       <c r="L147">
-        <v>0.652324444444444</v>
+        <v>0.65232444444444448</v>
       </c>
       <c r="M147">
         <v>1.12</v>
@@ -13095,7 +13095,7 @@
         </is>
       </c>
       <c r="L149">
-        <v>0.347653333333333</v>
+        <v>0.34765333333333337</v>
       </c>
       <c r="M149">
         <v>1.12</v>
@@ -13185,7 +13185,7 @@
         </is>
       </c>
       <c r="L150">
-        <v>0.444066666666667</v>
+        <v>0.44406666666666672</v>
       </c>
       <c r="M150">
         <v>1.12</v>
@@ -13275,7 +13275,7 @@
         </is>
       </c>
       <c r="L151">
-        <v>0.588515555555556</v>
+        <v>0.58851555555555557</v>
       </c>
       <c r="M151">
         <v>1.12</v>
@@ -13455,7 +13455,7 @@
         </is>
       </c>
       <c r="L153">
-        <v>0.555693333333333</v>
+        <v>0.55569333333333337</v>
       </c>
       <c r="M153">
         <v>1.12</v>
@@ -13635,7 +13635,7 @@
         </is>
       </c>
       <c r="L155">
-        <v>0.64884</v>
+        <v>0.64884000000000008</v>
       </c>
       <c r="M155">
         <v>1.12</v>
@@ -13725,7 +13725,7 @@
         </is>
       </c>
       <c r="L156">
-        <v>0.838524444444445</v>
+        <v>0.83852444444444463</v>
       </c>
       <c r="M156">
         <v>1.12</v>
@@ -13815,7 +13815,7 @@
         </is>
       </c>
       <c r="L157">
-        <v>0.473342222222222</v>
+        <v>0.47334222222222228</v>
       </c>
       <c r="M157">
         <v>1.12</v>
@@ -13965,7 +13965,7 @@
         </is>
       </c>
       <c r="L159">
-        <v>0.328364444444444</v>
+        <v>0.32836444444444446</v>
       </c>
       <c r="M159">
         <v>1.12</v>
@@ -14200,7 +14200,7 @@
         </is>
       </c>
       <c r="L162">
-        <v>0.446835555555556</v>
+        <v>0.4468355555555556</v>
       </c>
       <c r="M162">
         <v>1.12</v>
@@ -14380,7 +14380,7 @@
         </is>
       </c>
       <c r="L164">
-        <v>0.720737777777778</v>
+        <v>0.72073777777777792</v>
       </c>
       <c r="M164">
         <v>1.12</v>
@@ -14470,7 +14470,7 @@
         </is>
       </c>
       <c r="L165">
-        <v>0.566364444444444</v>
+        <v>0.56636444444444445</v>
       </c>
       <c r="M165">
         <v>1.12</v>
@@ -14560,7 +14560,7 @@
         </is>
       </c>
       <c r="L166">
-        <v>0.283782222222222</v>
+        <v>0.28378222222222227</v>
       </c>
       <c r="M166">
         <v>1.12</v>
@@ -14830,7 +14830,7 @@
         </is>
       </c>
       <c r="L169">
-        <v>0.647222222222222</v>
+        <v>0.64722222222222237</v>
       </c>
       <c r="M169">
         <v>1.12</v>
@@ -14920,7 +14920,7 @@
         </is>
       </c>
       <c r="L170">
-        <v>0.536031111111111</v>
+        <v>0.53603111111111112</v>
       </c>
       <c r="M170">
         <v>1.12</v>
@@ -15010,7 +15010,7 @@
         </is>
       </c>
       <c r="L171">
-        <v>0.416688888888889</v>
+        <v>0.41668888888888889</v>
       </c>
       <c r="M171">
         <v>1.12</v>
@@ -15100,7 +15100,7 @@
         </is>
       </c>
       <c r="L172">
-        <v>0.556128888888889</v>
+        <v>0.55612888888888889</v>
       </c>
       <c r="M172">
         <v>1.12</v>
@@ -15190,7 +15190,7 @@
         </is>
       </c>
       <c r="L173">
-        <v>0.425182222222222</v>
+        <v>0.42518222222222224</v>
       </c>
       <c r="M173">
         <v>1.12</v>
@@ -15280,7 +15280,7 @@
         </is>
       </c>
       <c r="L174">
-        <v>0.425182222222222</v>
+        <v>0.42518222222222224</v>
       </c>
       <c r="M174">
         <v>1.12</v>
@@ -15370,7 +15370,7 @@
         </is>
       </c>
       <c r="L175">
-        <v>0.416688888888889</v>
+        <v>0.41668888888888889</v>
       </c>
       <c r="M175">
         <v>1.12</v>
@@ -15460,7 +15460,7 @@
         </is>
       </c>
       <c r="L176">
-        <v>0.467306666666667</v>
+        <v>0.4673066666666667</v>
       </c>
       <c r="M176">
         <v>1.12</v>
@@ -15550,7 +15550,7 @@
         </is>
       </c>
       <c r="L177">
-        <v>1.06230666666667</v>
+        <v>1.0623066666666667</v>
       </c>
       <c r="M177">
         <v>1.12</v>
@@ -15640,7 +15640,7 @@
         </is>
       </c>
       <c r="L178">
-        <v>0.993706666666667</v>
+        <v>0.99370666666666685</v>
       </c>
       <c r="M178">
         <v>1.12</v>
@@ -15751,7 +15751,7 @@
         </is>
       </c>
       <c r="L179">
-        <v>1.44876888888889</v>
+        <v>1.448768888888889</v>
       </c>
       <c r="M179">
         <v>1.12</v>
@@ -15841,7 +15841,7 @@
         </is>
       </c>
       <c r="L180">
-        <v>0.362773333333333</v>
+        <v>0.36277333333333339</v>
       </c>
       <c r="M180">
         <v>1.12</v>
@@ -16021,7 +16021,7 @@
         </is>
       </c>
       <c r="L182">
-        <v>0.670493333333333</v>
+        <v>0.67049333333333339</v>
       </c>
       <c r="M182">
         <v>1.12</v>
@@ -16111,7 +16111,7 @@
         </is>
       </c>
       <c r="L183">
-        <v>0.308204444444445</v>
+        <v>0.3082044444444445</v>
       </c>
       <c r="M183">
         <v>1.12</v>
@@ -16341,7 +16341,7 @@
         </is>
       </c>
       <c r="L186">
-        <v>0.304564444444444</v>
+        <v>0.30456444444444447</v>
       </c>
       <c r="M186">
         <v>1.12</v>
@@ -16496,7 +16496,7 @@
         </is>
       </c>
       <c r="L188">
-        <v>0.503924444444445</v>
+        <v>0.50392444444444451</v>
       </c>
       <c r="M188">
         <v>1.12</v>
@@ -16586,7 +16586,7 @@
         </is>
       </c>
       <c r="L189">
-        <v>0.407324444444444</v>
+        <v>0.40732444444444449</v>
       </c>
       <c r="M189">
         <v>1.12</v>
@@ -16676,7 +16676,7 @@
         </is>
       </c>
       <c r="L190">
-        <v>0.304564444444444</v>
+        <v>0.30456444444444447</v>
       </c>
       <c r="M190">
         <v>1.12</v>
@@ -16836,7 +16836,7 @@
         </is>
       </c>
       <c r="L192">
-        <v>3.53132</v>
+        <v>3.5313200000000005</v>
       </c>
       <c r="M192">
         <v>1.12</v>
@@ -16947,7 +16947,7 @@
         </is>
       </c>
       <c r="L193">
-        <v>0.678644444444445</v>
+        <v>0.67864444444444461</v>
       </c>
       <c r="M193">
         <v>1.12</v>
@@ -17037,7 +17037,7 @@
         </is>
       </c>
       <c r="L194">
-        <v>0.395688888888889</v>
+        <v>0.39568888888888892</v>
       </c>
       <c r="M194">
         <v>1.12</v>
@@ -17127,7 +17127,7 @@
         </is>
       </c>
       <c r="L195">
-        <v>0.514564444444444</v>
+        <v>0.51456444444444449</v>
       </c>
       <c r="M195">
         <v>1.12</v>
@@ -17217,7 +17217,7 @@
         </is>
       </c>
       <c r="L196">
-        <v>0.395688888888889</v>
+        <v>0.39568888888888892</v>
       </c>
       <c r="M196">
         <v>1.12</v>
@@ -17307,7 +17307,7 @@
         </is>
       </c>
       <c r="L197">
-        <v>0.395688888888889</v>
+        <v>0.39568888888888892</v>
       </c>
       <c r="M197">
         <v>1.12</v>
@@ -17647,7 +17647,7 @@
         </is>
       </c>
       <c r="L201">
-        <v>0.354373333333333</v>
+        <v>0.35437333333333337</v>
       </c>
       <c r="M201">
         <v>1.12</v>
@@ -17737,7 +17737,7 @@
         </is>
       </c>
       <c r="L202">
-        <v>0.718248888888889</v>
+        <v>0.71824888888888894</v>
       </c>
       <c r="M202">
         <v>1.12</v>
@@ -17917,7 +17917,7 @@
         </is>
       </c>
       <c r="L204">
-        <v>0.438902222222222</v>
+        <v>0.43890222222222225</v>
       </c>
       <c r="M204">
         <v>1.12</v>
@@ -18007,7 +18007,7 @@
         </is>
       </c>
       <c r="L205">
-        <v>0.354373333333333</v>
+        <v>0.35437333333333337</v>
       </c>
       <c r="M205">
         <v>1.12</v>
@@ -18277,7 +18277,7 @@
         </is>
       </c>
       <c r="L208">
-        <v>0.622706666666667</v>
+        <v>0.62270666666666674</v>
       </c>
       <c r="M208">
         <v>1.12</v>
@@ -18367,7 +18367,7 @@
         </is>
       </c>
       <c r="L209">
-        <v>0.312964444444444</v>
+        <v>0.31296444444444449</v>
       </c>
       <c r="M209">
         <v>1.12</v>
@@ -18457,7 +18457,7 @@
         </is>
       </c>
       <c r="L210">
-        <v>17.6047411111111</v>
+        <v>17.60474111111111</v>
       </c>
       <c r="M210">
         <v>1.18</v>
@@ -18568,7 +18568,7 @@
         </is>
       </c>
       <c r="L211">
-        <v>0.527786666666667</v>
+        <v>0.52778666666666663</v>
       </c>
       <c r="M211">
         <v>1.12</v>
@@ -18658,7 +18658,7 @@
         </is>
       </c>
       <c r="L212">
-        <v>18.3532666666667</v>
+        <v>18.35326666666667</v>
       </c>
       <c r="M212">
         <v>1.12</v>
@@ -18769,7 +18769,7 @@
         </is>
       </c>
       <c r="L213">
-        <v>14.9398444444444</v>
+        <v>14.939844444444446</v>
       </c>
       <c r="M213">
         <v>1.12</v>
@@ -18880,7 +18880,7 @@
         </is>
       </c>
       <c r="L214">
-        <v>0.312964444444444</v>
+        <v>0.31296444444444449</v>
       </c>
       <c r="M214">
         <v>1.12</v>
@@ -18970,7 +18970,7 @@
         </is>
       </c>
       <c r="L215">
-        <v>0.362991111111111</v>
+        <v>0.3629911111111111</v>
       </c>
       <c r="M215">
         <v>1.12</v>
@@ -19060,7 +19060,7 @@
         </is>
       </c>
       <c r="L216">
-        <v>0.397182222222222</v>
+        <v>0.39718222222222221</v>
       </c>
       <c r="M216">
         <v>1.12</v>
@@ -19150,7 +19150,7 @@
         </is>
       </c>
       <c r="L217">
-        <v>0.372013333333333</v>
+        <v>0.37201333333333331</v>
       </c>
       <c r="M217">
         <v>1.12</v>
@@ -19330,7 +19330,7 @@
         </is>
       </c>
       <c r="L219">
-        <v>0.646288888888889</v>
+        <v>0.64628888888888891</v>
       </c>
       <c r="M219">
         <v>1.12</v>
@@ -19420,7 +19420,7 @@
         </is>
       </c>
       <c r="L220">
-        <v>0.355088888888889</v>
+        <v>0.3550888888888889</v>
       </c>
       <c r="M220">
         <v>1.12</v>
@@ -19600,7 +19600,7 @@
         </is>
       </c>
       <c r="L222">
-        <v>0.427733333333333</v>
+        <v>0.42773333333333341</v>
       </c>
       <c r="M222">
         <v>1.12</v>
@@ -19690,7 +19690,7 @@
         </is>
       </c>
       <c r="L223">
-        <v>0.355088888888889</v>
+        <v>0.3550888888888889</v>
       </c>
       <c r="M223">
         <v>1.12</v>
@@ -19780,7 +19780,7 @@
         </is>
       </c>
       <c r="L224">
-        <v>0.484386666666667</v>
+        <v>0.48438666666666674</v>
       </c>
       <c r="M224">
         <v>1.12</v>
@@ -19870,7 +19870,7 @@
         </is>
       </c>
       <c r="L225">
-        <v>0.371484444444445</v>
+        <v>0.37148444444444451</v>
       </c>
       <c r="M225">
         <v>1.12</v>
@@ -20050,7 +20050,7 @@
         </is>
       </c>
       <c r="L227">
-        <v>18.3342577777778</v>
+        <v>18.334257777777779</v>
       </c>
       <c r="M227">
         <v>1.12</v>
@@ -20251,7 +20251,7 @@
         </is>
       </c>
       <c r="L229">
-        <v>0.330946666666667</v>
+        <v>0.33094666666666667</v>
       </c>
       <c r="M229">
         <v>1.12</v>
@@ -20341,7 +20341,7 @@
         </is>
       </c>
       <c r="L230">
-        <v>0.483391111111111</v>
+        <v>0.48339111111111122</v>
       </c>
       <c r="M230">
         <v>1.12</v>
@@ -20501,7 +20501,7 @@
         </is>
       </c>
       <c r="L232">
-        <v>0.441048888888889</v>
+        <v>0.44104888888888893</v>
       </c>
       <c r="M232">
         <v>1.12</v>
@@ -20591,7 +20591,7 @@
         </is>
       </c>
       <c r="L233">
-        <v>0.304564444444444</v>
+        <v>0.30456444444444447</v>
       </c>
       <c r="M233">
         <v>1.12</v>
@@ -20681,7 +20681,7 @@
         </is>
       </c>
       <c r="L234">
-        <v>0.483391111111111</v>
+        <v>0.48339111111111122</v>
       </c>
       <c r="M234">
         <v>1.12</v>
@@ -20771,7 +20771,7 @@
         </is>
       </c>
       <c r="L235">
-        <v>0.592715555555556</v>
+        <v>0.59271555555555566</v>
       </c>
       <c r="M235">
         <v>1.12</v>
@@ -20931,7 +20931,7 @@
         </is>
       </c>
       <c r="L237">
-        <v>0.503924444444445</v>
+        <v>0.50392444444444451</v>
       </c>
       <c r="M237">
         <v>1.12</v>
@@ -21021,7 +21021,7 @@
         </is>
       </c>
       <c r="L238">
-        <v>0.407324444444444</v>
+        <v>0.40732444444444449</v>
       </c>
       <c r="M238">
         <v>1.12</v>
@@ -21111,7 +21111,7 @@
         </is>
       </c>
       <c r="L239">
-        <v>0.841946666666667</v>
+        <v>0.84194666666666684</v>
       </c>
       <c r="M239">
         <v>1.12</v>
@@ -21381,7 +21381,7 @@
         </is>
       </c>
       <c r="L242">
-        <v>6.03441666666667</v>
+        <v>6.034416666666667</v>
       </c>
       <c r="M242">
         <v>1.5</v>
@@ -21651,7 +21651,7 @@
         </is>
       </c>
       <c r="L245">
-        <v>1.32706222222222</v>
+        <v>1.3270622222222224</v>
       </c>
       <c r="M245">
         <v>1.12</v>
@@ -21741,7 +21741,7 @@
         </is>
       </c>
       <c r="L246">
-        <v>0.354311111111111</v>
+        <v>0.35431111111111113</v>
       </c>
       <c r="M246">
         <v>1.12</v>
@@ -21901,7 +21901,7 @@
         </is>
       </c>
       <c r="L248">
-        <v>0.354311111111111</v>
+        <v>0.35431111111111113</v>
       </c>
       <c r="M248">
         <v>1.12</v>
@@ -21991,7 +21991,7 @@
         </is>
       </c>
       <c r="L249">
-        <v>1.22078666666667</v>
+        <v>1.2207866666666669</v>
       </c>
       <c r="M249">
         <v>1.12</v>
@@ -22081,7 +22081,7 @@
         </is>
       </c>
       <c r="L250">
-        <v>0.354311111111111</v>
+        <v>0.35431111111111113</v>
       </c>
       <c r="M250">
         <v>1.12</v>
@@ -22171,7 +22171,7 @@
         </is>
       </c>
       <c r="L251">
-        <v>0.354311111111111</v>
+        <v>0.35431111111111113</v>
       </c>
       <c r="M251">
         <v>1.12</v>
@@ -22261,7 +22261,7 @@
         </is>
       </c>
       <c r="L252">
-        <v>0.354311111111111</v>
+        <v>0.35431111111111113</v>
       </c>
       <c r="M252">
         <v>1.12</v>
@@ -22351,7 +22351,7 @@
         </is>
       </c>
       <c r="L253">
-        <v>0.354311111111111</v>
+        <v>0.35431111111111113</v>
       </c>
       <c r="M253">
         <v>1.12</v>
@@ -22392,16 +22392,16 @@
     </row>
     <row r="254">
       <c r="A254">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOSPITAL CARLOS MONGE MEDRANO</t>
+          <t xml:space="preserve">HOSPITAL REGIONAL MANUEL NUÑEZ BUTRON</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t xml:space="preserve">3299</t>
+          <t xml:space="preserve">3251</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
@@ -22411,48 +22411,48 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t xml:space="preserve">“SANTA MARIA DE NIEVA”</t>
+          <t xml:space="preserve">HOSPITAL REGIONAL MANUEL NUÑEZ BUTRON</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t xml:space="preserve">5145</t>
+          <t xml:space="preserve">3251</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
         <is>
-          <t xml:space="preserve">I A</t>
+          <t xml:space="preserve">II</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t xml:space="preserve">AMAZONAS</t>
+          <t xml:space="preserve">PUNO</t>
         </is>
       </c>
       <c r="I254">
-        <v>1478.7</v>
+        <v>0</v>
       </c>
       <c r="J254">
-        <v>2545.6</v>
+        <v>0</v>
       </c>
       <c r="K254" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 d 5 h</t>
+          <t xml:space="preserve">12 min</t>
         </is>
       </c>
       <c r="L254">
-        <v>53.821175</v>
+        <v>0.2</v>
       </c>
       <c r="M254">
-        <v>1.35</v>
+        <v>1.5</v>
       </c>
       <c r="N254" t="inlineStr">
         <is>
-          <t xml:space="preserve">paso de altura</t>
+          <t xml:space="preserve">sierra alta sostenida</t>
         </is>
       </c>
       <c r="O254">
-        <v>4406</v>
+        <v>3841</v>
       </c>
       <c r="P254" t="inlineStr">
         <is>
@@ -22461,34 +22461,13 @@
       </c>
       <c r="R254" t="inlineStr">
         <is>
-          <t xml:space="preserve">si</t>
-        </is>
-      </c>
-      <c r="S254" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Juliaca (JUL)</t>
-        </is>
-      </c>
-      <c r="T254" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Jaén (JAE)</t>
-        </is>
-      </c>
-      <c r="U254" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LIM</t>
-        </is>
-      </c>
-      <c r="V254">
-        <v>1581</v>
-      </c>
-      <c r="W254" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9 h 08 min</t>
-        </is>
-      </c>
-      <c r="X254">
-        <v>9.13</v>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="Y254" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
+        </is>
       </c>
       <c r="Z254" t="inlineStr">
         <is>
@@ -22503,7 +22482,7 @@
     </row>
     <row r="255">
       <c r="A255">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B255" t="inlineStr">
         <is>
@@ -22522,17 +22501,17 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOSPITAL REGIONAL MANUEL NUÑEZ BUTRON</t>
+          <t xml:space="preserve">Hospital de Apoyo Ilave</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t xml:space="preserve">3251</t>
+          <t xml:space="preserve">3032</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
         <is>
-          <t xml:space="preserve">II</t>
+          <t xml:space="preserve">IA</t>
         </is>
       </c>
       <c r="H255" t="inlineStr">
@@ -22540,60 +22519,40 @@
           <t xml:space="preserve">PUNO</t>
         </is>
       </c>
-      <c r="I255">
-        <v>0</v>
-      </c>
-      <c r="J255">
-        <v>0</v>
-      </c>
-      <c r="K255" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12 min</t>
-        </is>
-      </c>
-      <c r="L255">
-        <v>0.2</v>
-      </c>
-      <c r="M255">
-        <v>1.5</v>
-      </c>
-      <c r="N255" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sierra alta sostenida</t>
-        </is>
-      </c>
-      <c r="O255">
-        <v>3841</v>
-      </c>
       <c r="P255" t="inlineStr">
         <is>
-          <t xml:space="preserve">sí</t>
+          <t xml:space="preserve">sin dato</t>
+        </is>
+      </c>
+      <c r="Q255" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Receptor sin ubicacion en el registro nacional de bancos de sangre</t>
         </is>
       </c>
       <c r="R255" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">sin dato</t>
         </is>
       </c>
       <c r="Y255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
+          <t xml:space="preserve">Receptor sin ubicacion en el registro</t>
         </is>
       </c>
       <c r="Z255" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">sin dato</t>
         </is>
       </c>
       <c r="AA255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sin puerto fluvial navegable a &lt;=150 km de algun extremo; acceso por carretera</t>
+          <t xml:space="preserve">Receptor sin ubicacion en el registro</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B256" t="inlineStr">
         <is>
@@ -22612,12 +22571,12 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hospital de Apoyo Ilave</t>
+          <t xml:space="preserve">Hospital II-1 "Rafael Ortiz Ravinez"</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t xml:space="preserve">3032</t>
+          <t xml:space="preserve">2990</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -22663,7 +22622,7 @@
     </row>
     <row r="257">
       <c r="A257">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B257" t="inlineStr">
         <is>
@@ -22682,17 +22641,17 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hospital II-1 "Rafael Ortiz Ravinez"</t>
+          <t xml:space="preserve">“CLINICA AMERICANA DE JULIACA”</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t xml:space="preserve">2990</t>
+          <t xml:space="preserve">10815</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
         <is>
-          <t xml:space="preserve">IA</t>
+          <t xml:space="preserve">I A</t>
         </is>
       </c>
       <c r="H257" t="inlineStr">
@@ -22700,40 +22659,60 @@
           <t xml:space="preserve">PUNO</t>
         </is>
       </c>
+      <c r="I257">
+        <v>39.5</v>
+      </c>
+      <c r="J257">
+        <v>42.9</v>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 h 19 min</t>
+        </is>
+      </c>
+      <c r="L257">
+        <v>1.3214583333333332</v>
+      </c>
+      <c r="M257">
+        <v>1.5</v>
+      </c>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sierra alta sostenida</t>
+        </is>
+      </c>
+      <c r="O257">
+        <v>3988</v>
+      </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t xml:space="preserve">sin dato</t>
-        </is>
-      </c>
-      <c r="Q257" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Receptor sin ubicacion en el registro nacional de bancos de sangre</t>
+          <t xml:space="preserve">sí</t>
         </is>
       </c>
       <c r="R257" t="inlineStr">
         <is>
-          <t xml:space="preserve">sin dato</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="Y257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Receptor sin ubicacion en el registro</t>
+          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
         </is>
       </c>
       <c r="Z257" t="inlineStr">
         <is>
-          <t xml:space="preserve">sin dato</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="AA257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Receptor sin ubicacion en el registro</t>
+          <t xml:space="preserve">Sin puerto fluvial navegable a &lt;=150 km de algun extremo; acceso por carretera</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B258" t="inlineStr">
         <is>
@@ -22752,17 +22731,17 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t xml:space="preserve">“CLINICA AMERICANA DE JULIACA”</t>
+          <t xml:space="preserve">Hospital Carlos Cornejo Rosello Vizcardo - Azángaro</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t xml:space="preserve">10815</t>
+          <t xml:space="preserve">2941</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
         <is>
-          <t xml:space="preserve">I A</t>
+          <t xml:space="preserve">IA</t>
         </is>
       </c>
       <c r="H258" t="inlineStr">
@@ -22770,60 +22749,40 @@
           <t xml:space="preserve">PUNO</t>
         </is>
       </c>
-      <c r="I258">
-        <v>39.5</v>
-      </c>
-      <c r="J258">
-        <v>42.9</v>
-      </c>
-      <c r="K258" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1 h 19 min</t>
-        </is>
-      </c>
-      <c r="L258">
-        <v>1.32145833333333</v>
-      </c>
-      <c r="M258">
-        <v>1.5</v>
-      </c>
-      <c r="N258" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sierra alta sostenida</t>
-        </is>
-      </c>
-      <c r="O258">
-        <v>3988</v>
-      </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t xml:space="preserve">sí</t>
+          <t xml:space="preserve">sin dato</t>
+        </is>
+      </c>
+      <c r="Q258" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Receptor sin ubicacion en el registro nacional de bancos de sangre</t>
         </is>
       </c>
       <c r="R258" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">sin dato</t>
         </is>
       </c>
       <c r="Y258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
+          <t xml:space="preserve">Receptor sin ubicacion en el registro</t>
         </is>
       </c>
       <c r="Z258" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
+          <t xml:space="preserve">sin dato</t>
         </is>
       </c>
       <c r="AA258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sin puerto fluvial navegable a &lt;=150 km de algun extremo; acceso por carretera</t>
+          <t xml:space="preserve">Receptor sin ubicacion en el registro</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B259" t="inlineStr">
         <is>
@@ -22842,12 +22801,12 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hospital Carlos Cornejo Rosello Vizcardo - Azángaro</t>
+          <t xml:space="preserve">Hospital II-2 San Martín de Porres Macusani" - Red Carabaya</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t xml:space="preserve">2941</t>
+          <t xml:space="preserve">2974</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -22893,77 +22852,118 @@
     </row>
     <row r="260">
       <c r="A260">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOSPITAL REGIONAL MANUEL NUÑEZ BUTRON</t>
+          <t xml:space="preserve">BANCO DE SANGRE REGIONAL SAN MARTIN</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t xml:space="preserve">3251</t>
+          <t xml:space="preserve">20686</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t xml:space="preserve">PUNO</t>
+          <t xml:space="preserve">SAN MARTIN</t>
         </is>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hospital II-2 San Martín de Porres Macusani" - Red Carabaya</t>
+          <t xml:space="preserve">Nombre comercial: Centro Médico Daniel Alcides Carrión y razón social Clínica Daniel Alcides Carrión S.I.R.L.</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t xml:space="preserve">2974</t>
+          <t xml:space="preserve">8012</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
         <is>
-          <t xml:space="preserve">IA</t>
+          <t xml:space="preserve">I A</t>
         </is>
       </c>
       <c r="H260" t="inlineStr">
         <is>
-          <t xml:space="preserve">PUNO</t>
-        </is>
+          <t xml:space="preserve">SAN MARTIN</t>
+        </is>
+      </c>
+      <c r="I260">
+        <v>100.9</v>
+      </c>
+      <c r="J260">
+        <v>137.4</v>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2 h 28 min</t>
+        </is>
+      </c>
+      <c r="L260">
+        <v>2.4658844444444448</v>
+      </c>
+      <c r="M260">
+        <v>1.12</v>
+      </c>
+      <c r="N260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">costa / llano</t>
+        </is>
+      </c>
+      <c r="O260">
+        <v>1146</v>
       </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t xml:space="preserve">sin dato</t>
-        </is>
-      </c>
-      <c r="Q260" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Receptor sin ubicacion en el registro nacional de bancos de sangre</t>
+          <t xml:space="preserve">sí</t>
         </is>
       </c>
       <c r="R260" t="inlineStr">
         <is>
-          <t xml:space="preserve">sin dato</t>
-        </is>
-      </c>
-      <c r="Y260" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Receptor sin ubicacion en el registro</t>
-        </is>
+          <t xml:space="preserve">si</t>
+        </is>
+      </c>
+      <c r="S260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarapoto (TPP)</t>
+        </is>
+      </c>
+      <c r="T260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rioja (RIJ)</t>
+        </is>
+      </c>
+      <c r="U260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LIM</t>
+        </is>
+      </c>
+      <c r="V260">
+        <v>1280</v>
+      </c>
+      <c r="W260" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 h 10 min</t>
+        </is>
+      </c>
+      <c r="X260">
+        <v>5.16</v>
       </c>
       <c r="Z260" t="inlineStr">
         <is>
-          <t xml:space="preserve">sin dato</t>
+          <t xml:space="preserve">no</t>
         </is>
       </c>
       <c r="AA260" t="inlineStr">
         <is>
-          <t xml:space="preserve">Receptor sin ubicacion en el registro</t>
+          <t xml:space="preserve">Origen y destino usan el mismo puerto fluvial; acceso por carretera</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B261" t="inlineStr">
         <is>
@@ -22982,12 +22982,12 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nombre comercial: Centro Médico Daniel Alcides Carrión y razón social Clínica Daniel Alcides Carrión S.I.R.L.</t>
+          <t xml:space="preserve">Razón Social Servicios Médicos Lionel Flores e Hijos S.A.C - Clinica San Martin</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t xml:space="preserve">8012</t>
+          <t xml:space="preserve">8269</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
@@ -23001,18 +23001,18 @@
         </is>
       </c>
       <c r="I261">
-        <v>100.9</v>
+        <v>0</v>
       </c>
       <c r="J261">
-        <v>137.4</v>
+        <v>0</v>
       </c>
       <c r="K261" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 h 28 min</t>
+          <t xml:space="preserve">12 min</t>
         </is>
       </c>
       <c r="L261">
-        <v>2.46588444444444</v>
+        <v>0.2</v>
       </c>
       <c r="M261">
         <v>1.12</v>
@@ -23023,7 +23023,7 @@
         </is>
       </c>
       <c r="O261">
-        <v>1146</v>
+        <v>337</v>
       </c>
       <c r="P261" t="inlineStr">
         <is>
@@ -23032,34 +23032,13 @@
       </c>
       <c r="R261" t="inlineStr">
         <is>
-          <t xml:space="preserve">si</t>
-        </is>
-      </c>
-      <c r="S261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tarapoto (TPP)</t>
-        </is>
-      </c>
-      <c r="T261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rioja (RIJ)</t>
-        </is>
-      </c>
-      <c r="U261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LIM</t>
-        </is>
-      </c>
-      <c r="V261">
-        <v>1280</v>
-      </c>
-      <c r="W261" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 h 10 min</t>
-        </is>
-      </c>
-      <c r="X261">
-        <v>5.16</v>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="Y261" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
+        </is>
       </c>
       <c r="Z261" t="inlineStr">
         <is>
@@ -23074,7 +23053,7 @@
     </row>
     <row r="262">
       <c r="A262">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B262" t="inlineStr">
         <is>
@@ -23093,12 +23072,12 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t xml:space="preserve">Razón Social Servicios Médicos Lionel Flores e Hijos S.A.C - Clinica San Martin</t>
+          <t xml:space="preserve">RURAL SAPOSOA - OFICINA DE GESTIÓN DE SERVICIOS DE SALUD HUALLAGA CENTRAL</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t xml:space="preserve">8269</t>
+          <t xml:space="preserve">6529</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
@@ -23112,18 +23091,18 @@
         </is>
       </c>
       <c r="I262">
-        <v>0</v>
+        <v>67.9</v>
       </c>
       <c r="J262">
-        <v>0</v>
+        <v>135.3</v>
       </c>
       <c r="K262" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 min</t>
+          <t xml:space="preserve">2 h 22 min</t>
         </is>
       </c>
       <c r="L262">
-        <v>0.2</v>
+        <v>2.3711511111111112</v>
       </c>
       <c r="M262">
         <v>1.12</v>
@@ -23134,7 +23113,7 @@
         </is>
       </c>
       <c r="O262">
-        <v>337</v>
+        <v>425</v>
       </c>
       <c r="P262" t="inlineStr">
         <is>
@@ -23164,7 +23143,7 @@
     </row>
     <row r="263">
       <c r="A263">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B263" t="inlineStr">
         <is>
@@ -23183,17 +23162,17 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t xml:space="preserve">RURAL SAPOSOA - OFICINA DE GESTIÓN DE SERVICIOS DE SALUD HUALLAGA CENTRAL</t>
+          <t xml:space="preserve">HOSPITAL MOYOBAMBA</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t xml:space="preserve">6529</t>
+          <t xml:space="preserve">6733</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t xml:space="preserve">I A</t>
+          <t xml:space="preserve">I C</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
@@ -23202,18 +23181,18 @@
         </is>
       </c>
       <c r="I263">
-        <v>67.9</v>
+        <v>84.4</v>
       </c>
       <c r="J263">
-        <v>135.3</v>
+        <v>114.1</v>
       </c>
       <c r="K263" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 h 22 min</t>
+          <t xml:space="preserve">2 h 05 min</t>
         </is>
       </c>
       <c r="L263">
-        <v>2.37115111111111</v>
+        <v>2.0871066666666667</v>
       </c>
       <c r="M263">
         <v>1.12</v>
@@ -23224,7 +23203,7 @@
         </is>
       </c>
       <c r="O263">
-        <v>425</v>
+        <v>1186</v>
       </c>
       <c r="P263" t="inlineStr">
         <is>
@@ -23233,13 +23212,34 @@
       </c>
       <c r="R263" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="Y263" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
-        </is>
+          <t xml:space="preserve">si</t>
+        </is>
+      </c>
+      <c r="S263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarapoto (TPP)</t>
+        </is>
+      </c>
+      <c r="T263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rioja (RIJ)</t>
+        </is>
+      </c>
+      <c r="U263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LIM</t>
+        </is>
+      </c>
+      <c r="V263">
+        <v>1280</v>
+      </c>
+      <c r="W263" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 h 35 min</t>
+        </is>
+      </c>
+      <c r="X263">
+        <v>5.59</v>
       </c>
       <c r="Z263" t="inlineStr">
         <is>
@@ -23254,7 +23254,7 @@
     </row>
     <row r="264">
       <c r="A264">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B264" t="inlineStr">
         <is>
@@ -23273,17 +23273,17 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOSPITAL MOYOBAMBA</t>
+          <t xml:space="preserve">HOSPITAL DE RIOJA</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t xml:space="preserve">6733</t>
+          <t xml:space="preserve">6732</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
         <is>
-          <t xml:space="preserve">I C</t>
+          <t xml:space="preserve">I B</t>
         </is>
       </c>
       <c r="H264" t="inlineStr">
@@ -23292,18 +23292,18 @@
         </is>
       </c>
       <c r="I264">
-        <v>84.4</v>
+        <v>100.9</v>
       </c>
       <c r="J264">
-        <v>114.1</v>
+        <v>137.4</v>
       </c>
       <c r="K264" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 h 05 min</t>
+          <t xml:space="preserve">2 h 28 min</t>
         </is>
       </c>
       <c r="L264">
-        <v>2.08710666666667</v>
+        <v>2.4658844444444448</v>
       </c>
       <c r="M264">
         <v>1.12</v>
@@ -23314,7 +23314,7 @@
         </is>
       </c>
       <c r="O264">
-        <v>1186</v>
+        <v>1146</v>
       </c>
       <c r="P264" t="inlineStr">
         <is>
@@ -23346,11 +23346,11 @@
       </c>
       <c r="W264" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 h 35 min</t>
+          <t xml:space="preserve">5 h 10 min</t>
         </is>
       </c>
       <c r="X264">
-        <v>5.59</v>
+        <v>5.16</v>
       </c>
       <c r="Z264" t="inlineStr">
         <is>
@@ -23365,7 +23365,7 @@
     </row>
     <row r="265">
       <c r="A265">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B265" t="inlineStr">
         <is>
@@ -23384,12 +23384,12 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOSPITAL DE RIOJA</t>
+          <t xml:space="preserve">HOSPITAL II E JUANJUI - M.C- LUIS IZQUIERDO VASQUEZ</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t xml:space="preserve">6732</t>
+          <t xml:space="preserve">6919</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
@@ -23403,18 +23403,18 @@
         </is>
       </c>
       <c r="I265">
-        <v>100.9</v>
+        <v>86.7</v>
       </c>
       <c r="J265">
-        <v>137.4</v>
+        <v>121.6</v>
       </c>
       <c r="K265" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 h 28 min</t>
+          <t xml:space="preserve">2 h 18 min</t>
         </is>
       </c>
       <c r="L265">
-        <v>2.46588444444444</v>
+        <v>2.3047911111111112</v>
       </c>
       <c r="M265">
         <v>1.12</v>
@@ -23425,7 +23425,7 @@
         </is>
       </c>
       <c r="O265">
-        <v>1146</v>
+        <v>428</v>
       </c>
       <c r="P265" t="inlineStr">
         <is>
@@ -23434,34 +23434,13 @@
       </c>
       <c r="R265" t="inlineStr">
         <is>
-          <t xml:space="preserve">si</t>
-        </is>
-      </c>
-      <c r="S265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tarapoto (TPP)</t>
-        </is>
-      </c>
-      <c r="T265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rioja (RIJ)</t>
-        </is>
-      </c>
-      <c r="U265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LIM</t>
-        </is>
-      </c>
-      <c r="V265">
-        <v>1280</v>
-      </c>
-      <c r="W265" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 h 10 min</t>
-        </is>
-      </c>
-      <c r="X265">
-        <v>5.16</v>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="Y265" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
+        </is>
       </c>
       <c r="Z265" t="inlineStr">
         <is>
@@ -23470,13 +23449,13 @@
       </c>
       <c r="AA265" t="inlineStr">
         <is>
-          <t xml:space="preserve">Origen y destino usan el mismo puerto fluvial; acceso por carretera</t>
+          <t xml:space="preserve">Sin puerto fluvial navegable a &lt;=150 km de algun extremo; acceso por carretera</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B266" t="inlineStr">
         <is>
@@ -23495,12 +23474,12 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOSPITAL II E JUANJUI - M.C- LUIS IZQUIERDO VASQUEZ</t>
+          <t xml:space="preserve">HOSPITAL II TARAPOTO - ESSALUD (SUSP TEMP)</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t xml:space="preserve">6919</t>
+          <t xml:space="preserve">27733</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -23514,18 +23493,18 @@
         </is>
       </c>
       <c r="I266">
-        <v>86.7</v>
+        <v>0</v>
       </c>
       <c r="J266">
-        <v>121.6</v>
+        <v>0</v>
       </c>
       <c r="K266" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 h 18 min</t>
+          <t xml:space="preserve">12 min</t>
         </is>
       </c>
       <c r="L266">
-        <v>2.30479111111111</v>
+        <v>0.2</v>
       </c>
       <c r="M266">
         <v>1.12</v>
@@ -23536,7 +23515,7 @@
         </is>
       </c>
       <c r="O266">
-        <v>428</v>
+        <v>337</v>
       </c>
       <c r="P266" t="inlineStr">
         <is>
@@ -23560,13 +23539,13 @@
       </c>
       <c r="AA266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sin puerto fluvial navegable a &lt;=150 km de algun extremo; acceso por carretera</t>
+          <t xml:space="preserve">Origen y destino usan el mismo puerto fluvial; acceso por carretera</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B267" t="inlineStr">
         <is>
@@ -23585,17 +23564,17 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOSPITAL II TARAPOTO - ESSALUD (SUSP TEMP)</t>
+          <t xml:space="preserve">HOSPITAL RURAL PICOTA</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t xml:space="preserve">27733</t>
+          <t xml:space="preserve">6457</t>
         </is>
       </c>
       <c r="G267" t="inlineStr">
         <is>
-          <t xml:space="preserve">I B</t>
+          <t xml:space="preserve">I A</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
@@ -23604,18 +23583,18 @@
         </is>
       </c>
       <c r="I267">
-        <v>0</v>
+        <v>48.2</v>
       </c>
       <c r="J267">
-        <v>0</v>
+        <v>60.2</v>
       </c>
       <c r="K267" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 min</t>
+          <t xml:space="preserve">1 h 12 min</t>
         </is>
       </c>
       <c r="L267">
-        <v>0.2</v>
+        <v>1.2061333333333333</v>
       </c>
       <c r="M267">
         <v>1.12</v>
@@ -23626,7 +23605,7 @@
         </is>
       </c>
       <c r="O267">
-        <v>337</v>
+        <v>440</v>
       </c>
       <c r="P267" t="inlineStr">
         <is>
@@ -23656,7 +23635,7 @@
     </row>
     <row r="268">
       <c r="A268">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B268" t="inlineStr">
         <is>
@@ -23675,12 +23654,12 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOSPITAL RURAL PICOTA</t>
+          <t xml:space="preserve">HOSPITAL TARAPOTO</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t xml:space="preserve">6457</t>
+          <t xml:space="preserve">6918</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -23694,18 +23673,18 @@
         </is>
       </c>
       <c r="I268">
-        <v>48.2</v>
+        <v>0</v>
       </c>
       <c r="J268">
-        <v>60.2</v>
+        <v>0</v>
       </c>
       <c r="K268" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 h 12 min</t>
+          <t xml:space="preserve">12 min</t>
         </is>
       </c>
       <c r="L268">
-        <v>1.20613333333333</v>
+        <v>0.2</v>
       </c>
       <c r="M268">
         <v>1.12</v>
@@ -23716,7 +23695,7 @@
         </is>
       </c>
       <c r="O268">
-        <v>440</v>
+        <v>337</v>
       </c>
       <c r="P268" t="inlineStr">
         <is>
@@ -23746,7 +23725,7 @@
     </row>
     <row r="269">
       <c r="A269">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B269" t="inlineStr">
         <is>
@@ -23765,12 +23744,12 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOSPITAL TARAPOTO</t>
+          <t xml:space="preserve">NC: CLINICA YANTALO - RS: CLINICA DOCENTE ADELINA SOPLIN SAC</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t xml:space="preserve">6918</t>
+          <t xml:space="preserve">23733</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
@@ -23784,18 +23763,18 @@
         </is>
       </c>
       <c r="I269">
-        <v>0</v>
+        <v>89.3</v>
       </c>
       <c r="J269">
-        <v>0</v>
+        <v>124.2</v>
       </c>
       <c r="K269" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 min</t>
+          <t xml:space="preserve">2 h 15 min</t>
         </is>
       </c>
       <c r="L269">
-        <v>0.2</v>
+        <v>2.2477955555555562</v>
       </c>
       <c r="M269">
         <v>1.12</v>
@@ -23806,7 +23785,7 @@
         </is>
       </c>
       <c r="O269">
-        <v>337</v>
+        <v>1186</v>
       </c>
       <c r="P269" t="inlineStr">
         <is>
@@ -23815,13 +23794,34 @@
       </c>
       <c r="R269" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="Y269" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
-        </is>
+          <t xml:space="preserve">si</t>
+        </is>
+      </c>
+      <c r="S269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarapoto (TPP)</t>
+        </is>
+      </c>
+      <c r="T269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rioja (RIJ)</t>
+        </is>
+      </c>
+      <c r="U269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LIM</t>
+        </is>
+      </c>
+      <c r="V269">
+        <v>1280</v>
+      </c>
+      <c r="W269" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 h 29 min</t>
+        </is>
+      </c>
+      <c r="X269">
+        <v>5.49</v>
       </c>
       <c r="Z269" t="inlineStr">
         <is>
@@ -23836,7 +23836,7 @@
     </row>
     <row r="270">
       <c r="A270">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B270" t="inlineStr">
         <is>
@@ -23855,12 +23855,12 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t xml:space="preserve">NC: CLINICA YANTALO - RS: CLINICA DOCENTE ADELINA SOPLIN SAC</t>
+          <t xml:space="preserve">CLINICA SINAI RS: SINAÍ INVESTMENTS &amp; HEALTH SOCIEDAD ANÓNIMA CERRADA – SINAÍ IH SAC</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t xml:space="preserve">23733</t>
+          <t xml:space="preserve">28254</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
@@ -23874,18 +23874,18 @@
         </is>
       </c>
       <c r="I270">
-        <v>89.3</v>
+        <v>100.9</v>
       </c>
       <c r="J270">
-        <v>124.2</v>
+        <v>137.4</v>
       </c>
       <c r="K270" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 h 15 min</t>
+          <t xml:space="preserve">2 h 28 min</t>
         </is>
       </c>
       <c r="L270">
-        <v>2.24779555555556</v>
+        <v>2.4658844444444448</v>
       </c>
       <c r="M270">
         <v>1.12</v>
@@ -23896,7 +23896,7 @@
         </is>
       </c>
       <c r="O270">
-        <v>1186</v>
+        <v>1146</v>
       </c>
       <c r="P270" t="inlineStr">
         <is>
@@ -23928,11 +23928,11 @@
       </c>
       <c r="W270" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 h 29 min</t>
+          <t xml:space="preserve">5 h 10 min</t>
         </is>
       </c>
       <c r="X270">
-        <v>5.49</v>
+        <v>5.16</v>
       </c>
       <c r="Z270" t="inlineStr">
         <is>
@@ -23947,7 +23947,7 @@
     </row>
     <row r="271">
       <c r="A271">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B271" t="inlineStr">
         <is>
@@ -23966,12 +23966,12 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLINICA SINAI RS: SINAÍ INVESTMENTS &amp; HEALTH SOCIEDAD ANÓNIMA CERRADA – SINAÍ IH SAC</t>
+          <t xml:space="preserve">Razon social Servic Medic Virgen de las Mercedes SAC NC Clinica Virgen de las Mercedes</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t xml:space="preserve">28254</t>
+          <t xml:space="preserve">26411</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
@@ -23985,18 +23985,18 @@
         </is>
       </c>
       <c r="I271">
-        <v>100.9</v>
+        <v>0</v>
       </c>
       <c r="J271">
-        <v>137.4</v>
+        <v>0</v>
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 h 28 min</t>
+          <t xml:space="preserve">12 min</t>
         </is>
       </c>
       <c r="L271">
-        <v>2.46588444444444</v>
+        <v>0.2</v>
       </c>
       <c r="M271">
         <v>1.12</v>
@@ -24007,7 +24007,7 @@
         </is>
       </c>
       <c r="O271">
-        <v>1146</v>
+        <v>337</v>
       </c>
       <c r="P271" t="inlineStr">
         <is>
@@ -24016,34 +24016,13 @@
       </c>
       <c r="R271" t="inlineStr">
         <is>
-          <t xml:space="preserve">si</t>
-        </is>
-      </c>
-      <c r="S271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tarapoto (TPP)</t>
-        </is>
-      </c>
-      <c r="T271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rioja (RIJ)</t>
-        </is>
-      </c>
-      <c r="U271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LIM</t>
-        </is>
-      </c>
-      <c r="V271">
-        <v>1280</v>
-      </c>
-      <c r="W271" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 h 10 min</t>
-        </is>
-      </c>
-      <c r="X271">
-        <v>5.16</v>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="Y271" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
+        </is>
       </c>
       <c r="Z271" t="inlineStr">
         <is>
@@ -24058,7 +24037,7 @@
     </row>
     <row r="272">
       <c r="A272">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B272" t="inlineStr">
         <is>
@@ -24077,12 +24056,12 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t xml:space="preserve">Razon social Servic Medic Virgen de las Mercedes SAC NC Clinica Virgen de las Mercedes</t>
+          <t xml:space="preserve">CENTRO MÉDICO TRINIDAD Y ESPECIALIDADES MÉDICAS</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t xml:space="preserve">26411</t>
+          <t xml:space="preserve">18606</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
@@ -24148,7 +24127,7 @@
     </row>
     <row r="273">
       <c r="A273">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B273" t="inlineStr">
         <is>
@@ -24167,12 +24146,12 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO MÉDICO TRINIDAD Y ESPECIALIDADES MÉDICAS</t>
+          <t xml:space="preserve">razón social SOLUMEDIC TARAPOTO S.A.C. y nombre comercial “SOLUCIONES MEDICAS SAN CAMILO”</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t xml:space="preserve">18606</t>
+          <t xml:space="preserve">34984</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
@@ -24238,7 +24217,7 @@
     </row>
     <row r="274">
       <c r="A274">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B274" t="inlineStr">
         <is>
@@ -24257,12 +24236,12 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t xml:space="preserve">razón social SOLUMEDIC TARAPOTO S.A.C. y nombre comercial “SOLUCIONES MEDICAS SAN CAMILO”</t>
+          <t xml:space="preserve">NC: CENTRO MEDICO LUZ DIVINA, RS: SERVICIOS MEDICOS LUZ DIVINA S.A.C.</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t xml:space="preserve">34984</t>
+          <t xml:space="preserve">28029</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
@@ -24276,18 +24255,18 @@
         </is>
       </c>
       <c r="I274">
-        <v>0</v>
+        <v>121.4</v>
       </c>
       <c r="J274">
-        <v>0</v>
+        <v>158.1</v>
       </c>
       <c r="K274" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 min</t>
+          <t xml:space="preserve">2 h 57 min</t>
         </is>
       </c>
       <c r="L274">
-        <v>0.2</v>
+        <v>2.9456222222222226</v>
       </c>
       <c r="M274">
         <v>1.12</v>
@@ -24298,7 +24277,7 @@
         </is>
       </c>
       <c r="O274">
-        <v>337</v>
+        <v>1129</v>
       </c>
       <c r="P274" t="inlineStr">
         <is>
@@ -24307,13 +24286,34 @@
       </c>
       <c r="R274" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="Y274" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
-        </is>
+          <t xml:space="preserve">si</t>
+        </is>
+      </c>
+      <c r="S274" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tarapoto (TPP)</t>
+        </is>
+      </c>
+      <c r="T274" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rioja (RIJ)</t>
+        </is>
+      </c>
+      <c r="U274" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LIM</t>
+        </is>
+      </c>
+      <c r="V274">
+        <v>1280</v>
+      </c>
+      <c r="W274" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5 h 33 min</t>
+        </is>
+      </c>
+      <c r="X274">
+        <v>5.55</v>
       </c>
       <c r="Z274" t="inlineStr">
         <is>
@@ -24328,7 +24328,7 @@
     </row>
     <row r="275">
       <c r="A275">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B275" t="inlineStr">
         <is>
@@ -24347,17 +24347,17 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t xml:space="preserve">NC: CENTRO MEDICO LUZ DIVINA, RS: SERVICIOS MEDICOS LUZ DIVINA S.A.C.</t>
+          <t xml:space="preserve">CENTRO NEUROQUIRURGICO DE LA SELVA S.A.C.-CLINICA RODRIGUEZ</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t xml:space="preserve">28029</t>
+          <t xml:space="preserve">32615</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t xml:space="preserve">I A</t>
+          <t xml:space="preserve">I B</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
@@ -24366,18 +24366,18 @@
         </is>
       </c>
       <c r="I275">
-        <v>121.4</v>
+        <v>0</v>
       </c>
       <c r="J275">
-        <v>158.1</v>
+        <v>0</v>
       </c>
       <c r="K275" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 h 57 min</t>
+          <t xml:space="preserve">12 min</t>
         </is>
       </c>
       <c r="L275">
-        <v>2.94562222222222</v>
+        <v>0.2</v>
       </c>
       <c r="M275">
         <v>1.12</v>
@@ -24388,7 +24388,7 @@
         </is>
       </c>
       <c r="O275">
-        <v>1129</v>
+        <v>337</v>
       </c>
       <c r="P275" t="inlineStr">
         <is>
@@ -24397,34 +24397,13 @@
       </c>
       <c r="R275" t="inlineStr">
         <is>
-          <t xml:space="preserve">si</t>
-        </is>
-      </c>
-      <c r="S275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tarapoto (TPP)</t>
-        </is>
-      </c>
-      <c r="T275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rioja (RIJ)</t>
-        </is>
-      </c>
-      <c r="U275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LIM</t>
-        </is>
-      </c>
-      <c r="V275">
-        <v>1280</v>
-      </c>
-      <c r="W275" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5 h 33 min</t>
-        </is>
-      </c>
-      <c r="X275">
-        <v>5.55</v>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="Y275" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
+        </is>
       </c>
       <c r="Z275" t="inlineStr">
         <is>
@@ -24439,7 +24418,7 @@
     </row>
     <row r="276">
       <c r="A276">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B276" t="inlineStr">
         <is>
@@ -24458,17 +24437,17 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO NEUROQUIRURGICO DE LA SELVA S.A.C.-CLINICA RODRIGUEZ</t>
+          <t xml:space="preserve">CENTRO MEDICO DE LA MUJER CORAZON DE JESUS - SERVICIOS MEDICOS Y DE EDUCACION PARA LA SALUD E.I.R.L.</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t xml:space="preserve">32615</t>
+          <t xml:space="preserve">18592</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t xml:space="preserve">I B</t>
+          <t xml:space="preserve">I A</t>
         </is>
       </c>
       <c r="H276" t="inlineStr">
@@ -24529,7 +24508,7 @@
     </row>
     <row r="277">
       <c r="A277">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B277" t="inlineStr">
         <is>
@@ -24548,12 +24527,12 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t xml:space="preserve">CENTRO MEDICO DE LA MUJER CORAZON DE JESUS - SERVICIOS MEDICOS Y DE EDUCACION PARA LA SALUD E.I.R.L.</t>
+          <t xml:space="preserve">HOSPITAL II-E BELLAVISTA</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t xml:space="preserve">18592</t>
+          <t xml:space="preserve">6502</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -24567,18 +24546,18 @@
         </is>
       </c>
       <c r="I277">
-        <v>0</v>
+        <v>67.8</v>
       </c>
       <c r="J277">
-        <v>0</v>
+        <v>95.8</v>
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t xml:space="preserve">12 min</t>
+          <t xml:space="preserve">1 h 40 min</t>
         </is>
       </c>
       <c r="L277">
-        <v>0.2</v>
+        <v>1.6600444444444444</v>
       </c>
       <c r="M277">
         <v>1.12</v>
@@ -24589,7 +24568,7 @@
         </is>
       </c>
       <c r="O277">
-        <v>337</v>
+        <v>446</v>
       </c>
       <c r="P277" t="inlineStr">
         <is>
@@ -24619,56 +24598,56 @@
     </row>
     <row r="278">
       <c r="A278">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t xml:space="preserve">BANCO DE SANGRE REGIONAL SAN MARTIN</t>
+          <t xml:space="preserve">HOSPITAL III DANIEL ALCIDES CARRION - SEGURO SOCIAL DE SALUD</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t xml:space="preserve">20686</t>
+          <t xml:space="preserve">10185</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAN MARTIN</t>
+          <t xml:space="preserve">TACNA</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t xml:space="preserve">HOSPITAL II-E BELLAVISTA</t>
+          <t xml:space="preserve">Hospital II Moquegua - EsSalud</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t xml:space="preserve">6502</t>
+          <t xml:space="preserve">16157</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t xml:space="preserve">I A</t>
+          <t xml:space="preserve">I C</t>
         </is>
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t xml:space="preserve">SAN MARTIN</t>
+          <t xml:space="preserve">MOQUEGUA</t>
         </is>
       </c>
       <c r="I278">
-        <v>67.8</v>
+        <v>114.4</v>
       </c>
       <c r="J278">
-        <v>95.8</v>
+        <v>169.9</v>
       </c>
       <c r="K278" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 h 40 min</t>
+          <t xml:space="preserve">3 h 36 min</t>
         </is>
       </c>
       <c r="L278">
-        <v>1.66004444444444</v>
+        <v>3.6081333333333339</v>
       </c>
       <c r="M278">
         <v>1.12</v>
@@ -24679,7 +24658,7 @@
         </is>
       </c>
       <c r="O278">
-        <v>446</v>
+        <v>1424</v>
       </c>
       <c r="P278" t="inlineStr">
         <is>
@@ -24688,13 +24667,34 @@
       </c>
       <c r="R278" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="Y278" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
-        </is>
+          <t xml:space="preserve">si</t>
+        </is>
+      </c>
+      <c r="S278" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tacna (TCQ)</t>
+        </is>
+      </c>
+      <c r="T278" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ilo (ILQ)</t>
+        </is>
+      </c>
+      <c r="U278" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LIM</t>
+        </is>
+      </c>
+      <c r="V278">
+        <v>1879</v>
+      </c>
+      <c r="W278" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7 h 42 min</t>
+        </is>
+      </c>
+      <c r="X278">
+        <v>7.7</v>
       </c>
       <c r="Z278" t="inlineStr">
         <is>
@@ -24703,146 +24703,42 @@
       </c>
       <c r="AA278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Origen y destino usan el mismo puerto fluvial; acceso por carretera</t>
+          <t xml:space="preserve">Sin puerto fluvial navegable a &lt;=150 km de algun extremo; acceso por carretera</t>
         </is>
       </c>
     </row>
     <row r="279">
-      <c r="A279">
-        <v>278</v>
-      </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HOSPITAL III DANIEL ALCIDES CARRION - SEGURO SOCIAL DE SALUD</t>
-        </is>
-      </c>
-      <c r="C279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10185</t>
-        </is>
-      </c>
-      <c r="D279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TACNA</t>
-        </is>
-      </c>
-      <c r="E279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Hospital II Moquegua - EsSalud</t>
-        </is>
-      </c>
-      <c r="F279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">16157</t>
-        </is>
-      </c>
-      <c r="G279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">I C</t>
-        </is>
-      </c>
-      <c r="H279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MOQUEGUA</t>
-        </is>
-      </c>
-      <c r="I279">
-        <v>114.4</v>
-      </c>
-      <c r="J279">
-        <v>169.9</v>
-      </c>
-      <c r="K279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3 h 36 min</t>
-        </is>
-      </c>
-      <c r="L279">
-        <v>3.60813333333333</v>
-      </c>
-      <c r="M279">
-        <v>1.12</v>
-      </c>
-      <c r="N279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">costa / llano</t>
-        </is>
-      </c>
-      <c r="O279">
-        <v>1424</v>
-      </c>
-      <c r="P279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">sí</t>
-        </is>
-      </c>
-      <c r="R279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">si</t>
-        </is>
-      </c>
-      <c r="S279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Tacna (TCQ)</t>
-        </is>
-      </c>
-      <c r="T279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ilo (ILQ)</t>
-        </is>
-      </c>
-      <c r="U279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LIM</t>
-        </is>
-      </c>
-      <c r="V279">
-        <v>1879</v>
-      </c>
-      <c r="W279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7 h 42 min</t>
-        </is>
-      </c>
-      <c r="X279">
-        <v>7.7</v>
-      </c>
-      <c r="Z279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="AA279" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sin puerto fluvial navegable a &lt;=150 km de algun extremo; acceso por carretera</t>
+      <c r="A279" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VIA TERRESTRE: ruta real de carretera (OSRM sobre OpenStreetMap) del banco productor tipo II al hospital receptor tipo I, con tiempo de manejo de auto particular corregido por altitud del trayecto (open-meteo) y margen por paradas.</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t xml:space="preserve">VIA TERRESTRE: ruta real de carretera (OSRM sobre OpenStreetMap) del banco productor tipo II al hospital receptor tipo I, con tiempo de manejo de auto particular corregido por altitud del trayecto (open-meteo) y margen por paradas.</t>
+          <t xml:space="preserve">VIA AEREA: solo se calcula cuando el origen y el destino usan aeropuertos distintos con servicio comercial. Aeropuerto mas cercano en cada extremo; vuelo directo si es ruta habitual, si no con escala en Lima. Tiempo puerta a puerta = traslado en tierra a/desde el aeropuerto + presentacion (45 min) + vuelo + escala.</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t xml:space="preserve">VIA AEREA: solo se calcula cuando el origen y el destino usan aeropuertos distintos con servicio comercial. Aeropuerto mas cercano en cada extremo; vuelo directo si es ruta habitual, si no con escala en Lima. Tiempo puerta a puerta = traslado en tierra a/desde el aeropuerto + presentacion (45 min) + vuelo + escala.</t>
+          <t xml:space="preserve">VIA ACUATICA (fluvial): se evalua contra la red curada de puertos navegables (APN/MTC); solo aplica si ambos extremos tienen un puerto navegable distinto a &lt;=150 km y existe ruta de rio entre ambos.</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t xml:space="preserve">VIA ACUATICA (fluvial): se evalua contra la red curada de puertos navegables (APN/MTC); solo aplica si ambos extremos tienen un puerto navegable distinto a &lt;=150 km y existe ruta de rio entre ambos.</t>
+          <t xml:space="preserve">"sin dato": el hospital receptor no figura con ubicacion en el Registro Nacional de Bancos de Sangre (su codigo RENIPRESS no esta en el registro).</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t xml:space="preserve">"sin dato": el hospital receptor no figura con ubicacion en el Registro Nacional de Bancos de Sangre (su codigo RENIPRESS no esta en el registro).</t>
+          <t xml:space="preserve">Convenio Hospital Carlos Monge Medrano (Puno, RENIPRESS 3299) -&gt; Santa Maria de Nieva (Amazonas, RENIPRESS 5145) retirado de la base y del aplicativo: el codigo RENIPRESS 3299 en la planilla semaforo corresponde en realidad al Hospital de Apoyo Gustavo Lanatta Lujan (fila eliminada de la fuente).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corregir codigo RENIPRESS del convenio Hospital Docente de Trujillo -> Clinica Camino Real
El receptor usaba RENIPRESS 34335 (Clinica Camino Real de San Isidro,
Lima), generando un convenio ficticio Trujillo-Lima de 559 km / 10 h
24. El codigo correcto es 16830 (RS: GPS Trujillo SAC y NC: Clinica
Camino Real, Trujillo, La Libertad): es un convenio intra-Trujillo.
Se regenera la red de convenios, el Excel de tiempos y la
presentacion resumen.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/Convenios_tiempos_ruta_BS2_a_BS1.xlsx
+++ b/datos/Convenios_tiempos_ruta_BS2_a_BS1.xlsx
@@ -8873,37 +8873,37 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLINICA CAMINO REAL</t>
+          <t xml:space="preserve">RS: GPS TRUJILLO SAC Y NC: CLINICA CAMINO REAL</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t xml:space="preserve">34335</t>
+          <t xml:space="preserve">16830</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t xml:space="preserve">I A</t>
+          <t xml:space="preserve">I B</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t xml:space="preserve">LIMA</t>
+          <t xml:space="preserve">LA LIBERTAD</t>
         </is>
       </c>
       <c r="I101">
-        <v>493.9</v>
+        <v>0</v>
       </c>
       <c r="J101">
-        <v>559.2</v>
+        <v>0</v>
       </c>
       <c r="K101" t="inlineStr">
         <is>
-          <t xml:space="preserve">10 h 24 min</t>
+          <t xml:space="preserve">12 min</t>
         </is>
       </c>
       <c r="L101">
-        <v>10.401471111111114</v>
+        <v>0.2</v>
       </c>
       <c r="M101">
         <v>1.12</v>
@@ -8914,7 +8914,7 @@
         </is>
       </c>
       <c r="O101">
-        <v>394</v>
+        <v>35</v>
       </c>
       <c r="P101" t="inlineStr">
         <is>
@@ -8923,34 +8923,13 @@
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t xml:space="preserve">si</t>
-        </is>
-      </c>
-      <c r="S101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Trujillo (TRU)</t>
-        </is>
-      </c>
-      <c r="T101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lima (LIM)</t>
-        </is>
-      </c>
-      <c r="U101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">directo</t>
-        </is>
-      </c>
-      <c r="V101">
-        <v>490</v>
-      </c>
-      <c r="W101" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2 h 38 min</t>
-        </is>
-      </c>
-      <c r="X101">
-        <v>2.63</v>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="Y101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Origen y destino comparten el mismo aeropuerto; el traslado es terrestre</t>
+        </is>
       </c>
       <c r="Z101" t="inlineStr">
         <is>
@@ -24745,19 +24724,26 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fuente de convenios: base semaforo actualizada (relacion por codigo RENIPRESS), recibida el </t>
+          <t xml:space="preserve">Convenio N100 corregido: Hospital Regional Docente de Trujillo -&gt; Clinica Camino Real. El RENIPRESS del receptor en la planilla semaforo era 34335 (Clinica Camino Real de San Isidro, Lima); el codigo correcto es 16830 (RS: GPS Trujillo SAC y NC: Clinica Camino Real, Trujillo, La Libertad). Corregido: convenio intra-Trujillo, ya no aparece via aerea.</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-04</t>
+          <t xml:space="preserve">Fuente de convenios: base semaforo actualizada (relacion por codigo RENIPRESS), recibida el </t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
         <is>
           <t xml:space="preserve">.</t>
         </is>

</xml_diff>